<commit_message>
docs(performance): HCM_12 UAT grown to Phase B — 44 cases (goal approval/competency/scoring)
Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/PRD/HCM_12_Performance_Management_Multi_Tenant_PRD/Performance_UAT_Test_Script.xlsx
+++ b/PRD/HCM_12_Performance_Management_Multi_Tenant_PRD/Performance_UAT_Test_Script.xlsx
@@ -585,7 +585,7 @@
       </c>
       <c r="C7" s="4" t="inlineStr">
         <is>
-          <t>Phase A (configuration foundation): rating scales with score bands (M388), review templates with weighted sections + cycle audience scoping (M389), KPI library + per-cycle assignments with automatic achievement/rating scoring (M390), OKR objectives + key results + check-ins with progress roll-up (M391).</t>
+          <t>Phase A (configuration foundation): rating scales with score bands (M388), review templates with weighted sections + cycle audience scoping (M389), KPI library + per-cycle assignments with automatic achievement/rating scoring (M390), OKR objectives + key results + check-ins with progress roll-up (M391). Phase B (goals &amp; scoring): goal-plan approval workflow Employee→Manager with weights-must-total-100 validation + progress-update audit trail (M392), per-review competency assessment with position-requirement seeding and gap analysis (M393), §18 weighted section scoring + score→band conversion + HR rating override with preserved original (M394).</t>
         </is>
       </c>
     </row>
@@ -636,7 +636,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G30"/>
+  <dimension ref="A1:G45"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -1526,9 +1526,444 @@
       <c r="F30" s="8" t="inlineStr"/>
       <c r="G30" s="7" t="inlineStr"/>
     </row>
+    <row r="31" ht="57" customHeight="1">
+      <c r="A31" s="9" t="inlineStr">
+        <is>
+          <t>GPL-01</t>
+        </is>
+      </c>
+      <c r="B31" s="10" t="inlineStr">
+        <is>
+          <t>Goal plan submit (M392)</t>
+        </is>
+      </c>
+      <c r="C31" s="10" t="inlineStr">
+        <is>
+          <t>HR Admin</t>
+        </is>
+      </c>
+      <c r="D31" s="10" t="inlineStr">
+        <is>
+          <t>Performance → Goals. Pick a cycle + ONE employee (who has a manager). Create 2 DRAFT goals with weights 60 and 30. Look at the 'weights' tag next to the filters.</t>
+        </is>
+      </c>
+      <c r="E31" s="10" t="inlineStr">
+        <is>
+          <t>The tag shows 'weights 90%' in red and 'Submit plan for approval' is disabled (weights must total exactly 100 — §37.5).</t>
+        </is>
+      </c>
+      <c r="F31" s="8" t="inlineStr"/>
+      <c r="G31" s="10" t="inlineStr"/>
+    </row>
+    <row r="32" ht="57" customHeight="1">
+      <c r="A32" s="6" t="inlineStr">
+        <is>
+          <t>GPL-02</t>
+        </is>
+      </c>
+      <c r="B32" s="7" t="inlineStr">
+        <is>
+          <t>Goal plan submit (M392)</t>
+        </is>
+      </c>
+      <c r="C32" s="7" t="inlineStr">
+        <is>
+          <t>HR Admin</t>
+        </is>
+      </c>
+      <c r="D32" s="7" t="inlineStr">
+        <is>
+          <t>Edit one goal's weight so the two total 100 (60+40). Click 'Submit plan for approval'.</t>
+        </is>
+      </c>
+      <c r="E32" s="7" t="inlineStr">
+        <is>
+          <t>The tag turns green at 100%; submission succeeds — both goals show Approval = PENDING APPROVAL and editing them is now blocked.</t>
+        </is>
+      </c>
+      <c r="F32" s="8" t="inlineStr"/>
+      <c r="G32" s="7" t="inlineStr"/>
+    </row>
+    <row r="33" ht="57" customHeight="1">
+      <c r="A33" s="9" t="inlineStr">
+        <is>
+          <t>GPL-03</t>
+        </is>
+      </c>
+      <c r="B33" s="10" t="inlineStr">
+        <is>
+          <t>Goal plan approve (M392)</t>
+        </is>
+      </c>
+      <c r="C33" s="10" t="inlineStr">
+        <is>
+          <t>Manager</t>
+        </is>
+      </c>
+      <c r="D33" s="10" t="inlineStr">
+        <is>
+          <t>Sign in as the employee's MANAGER → Approvals inbox. Find 'Goal plan: &lt;employee&gt; (2 goals, weights 100%)' and Approve it.</t>
+        </is>
+      </c>
+      <c r="E33" s="10" t="inlineStr">
+        <is>
+          <t>After approval the goals' Approval column shows APPROVED and their status flips DRAFT → ACTIVE.</t>
+        </is>
+      </c>
+      <c r="F33" s="8" t="inlineStr"/>
+      <c r="G33" s="10" t="inlineStr"/>
+    </row>
+    <row r="34" ht="42" customHeight="1">
+      <c r="A34" s="6" t="inlineStr">
+        <is>
+          <t>GPL-04</t>
+        </is>
+      </c>
+      <c r="B34" s="7" t="inlineStr">
+        <is>
+          <t>Goal plan reject (M392)</t>
+        </is>
+      </c>
+      <c r="C34" s="7" t="inlineStr">
+        <is>
+          <t>HR Admin / Manager</t>
+        </is>
+      </c>
+      <c r="D34" s="7" t="inlineStr">
+        <is>
+          <t>Create another employee's plan (weights = 100), submit, and as their manager REJECT it in the Approvals inbox.</t>
+        </is>
+      </c>
+      <c r="E34" s="7" t="inlineStr">
+        <is>
+          <t>Goals show Approval = REJECTED and stay DRAFT — they can be edited and resubmitted (rework loop).</t>
+        </is>
+      </c>
+      <c r="F34" s="8" t="inlineStr"/>
+      <c r="G34" s="7" t="inlineStr"/>
+    </row>
+    <row r="35" ht="57" customHeight="1">
+      <c r="A35" s="9" t="inlineStr">
+        <is>
+          <t>GPL-05</t>
+        </is>
+      </c>
+      <c r="B35" s="10" t="inlineStr">
+        <is>
+          <t>Approved-edit guard (M392)</t>
+        </is>
+      </c>
+      <c r="C35" s="10" t="inlineStr">
+        <is>
+          <t>HR Admin</t>
+        </is>
+      </c>
+      <c r="D35" s="10" t="inlineStr">
+        <is>
+          <t>Edit an APPROVED goal (change its title or weight). Save, then look at its Approval column.</t>
+        </is>
+      </c>
+      <c r="E35" s="10" t="inlineStr">
+        <is>
+          <t>The edit works but Approval drops back to '—' (NOT_SUBMITTED) — a structurally changed goal must be resubmitted for approval (traceable).</t>
+        </is>
+      </c>
+      <c r="F35" s="8" t="inlineStr"/>
+      <c r="G35" s="10" t="inlineStr"/>
+    </row>
+    <row r="36" ht="57" customHeight="1">
+      <c r="A36" s="6" t="inlineStr">
+        <is>
+          <t>GPT-01</t>
+        </is>
+      </c>
+      <c r="B36" s="7" t="inlineStr">
+        <is>
+          <t>Progress trail (M392)</t>
+        </is>
+      </c>
+      <c r="C36" s="7" t="inlineStr">
+        <is>
+          <t>HR Admin</t>
+        </is>
+      </c>
+      <c r="D36" s="7" t="inlineStr">
+        <is>
+          <t>On any ACTIVE goal click 'Progress', set 40% with note 'Q2 checkpoint', save. Update again to 70% with another note. Then click 'History'.</t>
+        </is>
+      </c>
+      <c r="E36" s="7" t="inlineStr">
+        <is>
+          <t>The drawer shows BOTH updates newest-first: 40% → 70% with old→new values, notes, who and when (§6.4 audit trail).</t>
+        </is>
+      </c>
+      <c r="F36" s="8" t="inlineStr"/>
+      <c r="G36" s="7" t="inlineStr"/>
+    </row>
+    <row r="37" ht="87" customHeight="1">
+      <c r="A37" s="9" t="inlineStr">
+        <is>
+          <t>CMP-01</t>
+        </is>
+      </c>
+      <c r="B37" s="10" t="inlineStr">
+        <is>
+          <t>Competency seed (M393)</t>
+        </is>
+      </c>
+      <c r="C37" s="10" t="inlineStr">
+        <is>
+          <t>HR Admin</t>
+        </is>
+      </c>
+      <c r="D37" s="10" t="inlineStr">
+        <is>
+          <t>Open a performance review (Performance → Reviews → any review). In the 'Competency assessment' card click 'Seed from position'. (The employee's position must have required competencies — set them under Staffing → Position requirements if empty.)</t>
+        </is>
+      </c>
+      <c r="E37" s="10" t="inlineStr">
+        <is>
+          <t>One row per required competency appears with the Required level snapshot. If the position has none, a clear message says to add manually instead.</t>
+        </is>
+      </c>
+      <c r="F37" s="8" t="inlineStr"/>
+      <c r="G37" s="10" t="inlineStr"/>
+    </row>
+    <row r="38" ht="57" customHeight="1">
+      <c r="A38" s="6" t="inlineStr">
+        <is>
+          <t>CMP-02</t>
+        </is>
+      </c>
+      <c r="B38" s="7" t="inlineStr">
+        <is>
+          <t>Competency add + assess (M393)</t>
+        </is>
+      </c>
+      <c r="C38" s="7" t="inlineStr">
+        <is>
+          <t>HR Admin</t>
+        </is>
+      </c>
+      <c r="D38" s="7" t="inlineStr">
+        <is>
+          <t>Click 'Add competency', pick one from the catalog with Required level 4. Then click 'Assess' on it: Self=3, Manager=3, Final=3, comment. Save.</t>
+        </is>
+      </c>
+      <c r="E38" s="7" t="inlineStr">
+        <is>
+          <t>The row shows levels 3/3/3 and Gap = '-1 below' in red (gap = required − final; positive gap = development need).</t>
+        </is>
+      </c>
+      <c r="F38" s="8" t="inlineStr"/>
+      <c r="G38" s="7" t="inlineStr"/>
+    </row>
+    <row r="39" ht="42" customHeight="1">
+      <c r="A39" s="9" t="inlineStr">
+        <is>
+          <t>CMP-03</t>
+        </is>
+      </c>
+      <c r="B39" s="10" t="inlineStr">
+        <is>
+          <t>Competency gap states (M393)</t>
+        </is>
+      </c>
+      <c r="C39" s="10" t="inlineStr">
+        <is>
+          <t>HR Admin</t>
+        </is>
+      </c>
+      <c r="D39" s="10" t="inlineStr">
+        <is>
+          <t>Assess another row with Final = required level, and one with Final ABOVE required.</t>
+        </is>
+      </c>
+      <c r="E39" s="10" t="inlineStr">
+        <is>
+          <t>Gap shows 'meets' (blue) when equal and '+N above' (green) when above.</t>
+        </is>
+      </c>
+      <c r="F39" s="8" t="inlineStr"/>
+      <c r="G39" s="10" t="inlineStr"/>
+    </row>
+    <row r="40" ht="42" customHeight="1">
+      <c r="A40" s="6" t="inlineStr">
+        <is>
+          <t>CMP-04</t>
+        </is>
+      </c>
+      <c r="B40" s="7" t="inlineStr">
+        <is>
+          <t>Duplicate guard (M393)</t>
+        </is>
+      </c>
+      <c r="C40" s="7" t="inlineStr">
+        <is>
+          <t>HR Admin</t>
+        </is>
+      </c>
+      <c r="D40" s="7" t="inlineStr">
+        <is>
+          <t>Try adding the SAME competency to the review again.</t>
+        </is>
+      </c>
+      <c r="E40" s="7" t="inlineStr">
+        <is>
+          <t>Rejected — the competency is already on the review (it's also hidden from the picker).</t>
+        </is>
+      </c>
+      <c r="F40" s="8" t="inlineStr"/>
+      <c r="G40" s="7" t="inlineStr"/>
+    </row>
+    <row r="41" ht="87" customHeight="1">
+      <c r="A41" s="9" t="inlineStr">
+        <is>
+          <t>SCR-01</t>
+        </is>
+      </c>
+      <c r="B41" s="10" t="inlineStr">
+        <is>
+          <t>Weighted scoring (M394)</t>
+        </is>
+      </c>
+      <c r="C41" s="10" t="inlineStr">
+        <is>
+          <t>HR Admin</t>
+        </is>
+      </c>
+      <c r="D41" s="10" t="inlineStr">
+        <is>
+          <t>On a review where goals are RATED (Goals page → Rate) and competencies have FINAL levels: in the 'Weighted scores (§18)' card enter Values score 4 and click 'Compute scores'.</t>
+        </is>
+      </c>
+      <c r="E41" s="10" t="inlineStr">
+        <is>
+          <t>Goal/KPI/Competency/Values cells populate; Overall = weighted average using the template weights (Goals 50 / KPI 25 / Competency 20 / Values 5), re-normalised over the sections that have scores; the §18.3 band label (e.g. 'Exceeds Expectations') appears next to it.</t>
+        </is>
+      </c>
+      <c r="F41" s="8" t="inlineStr"/>
+      <c r="G41" s="10" t="inlineStr"/>
+    </row>
+    <row r="42" ht="57" customHeight="1">
+      <c r="A42" s="6" t="inlineStr">
+        <is>
+          <t>SCR-02</t>
+        </is>
+      </c>
+      <c r="B42" s="7" t="inlineStr">
+        <is>
+          <t>Missing-section handling (M394)</t>
+        </is>
+      </c>
+      <c r="C42" s="7" t="inlineStr">
+        <is>
+          <t>HR Admin</t>
+        </is>
+      </c>
+      <c r="D42" s="7" t="inlineStr">
+        <is>
+          <t>Compute scores on a review with NO KPI assignments (KPI cell —).</t>
+        </is>
+      </c>
+      <c r="E42" s="7" t="inlineStr">
+        <is>
+          <t>The overall still computes — the missing KPI section is left out and the remaining weights are re-normalised (it is NOT dragged down by a zero).</t>
+        </is>
+      </c>
+      <c r="F42" s="8" t="inlineStr"/>
+      <c r="G42" s="7" t="inlineStr"/>
+    </row>
+    <row r="43" ht="57" customHeight="1">
+      <c r="A43" s="9" t="inlineStr">
+        <is>
+          <t>OVR-01</t>
+        </is>
+      </c>
+      <c r="B43" s="10" t="inlineStr">
+        <is>
+          <t>HR override (M394)</t>
+        </is>
+      </c>
+      <c r="C43" s="10" t="inlineStr">
+        <is>
+          <t>HR Admin</t>
+        </is>
+      </c>
+      <c r="D43" s="10" t="inlineStr">
+        <is>
+          <t>On the scored review click 'Override rating'. New rating=4.5, Reason='Calibration committee decision'. Confirm.</t>
+        </is>
+      </c>
+      <c r="E43" s="10" t="inlineStr">
+        <is>
+          <t>Final rating becomes 4.50 with an 'overridden' tag; the Override cell shows the ORIGINAL computed rating, who overrode and the reason (original preserved — §18.4).</t>
+        </is>
+      </c>
+      <c r="F43" s="8" t="inlineStr"/>
+      <c r="G43" s="10" t="inlineStr"/>
+    </row>
+    <row r="44" ht="42" customHeight="1">
+      <c r="A44" s="6" t="inlineStr">
+        <is>
+          <t>OVR-02</t>
+        </is>
+      </c>
+      <c r="B44" s="7" t="inlineStr">
+        <is>
+          <t>Override guards (M394)</t>
+        </is>
+      </c>
+      <c r="C44" s="7" t="inlineStr">
+        <is>
+          <t>HR Admin / HR Specialist</t>
+        </is>
+      </c>
+      <c r="D44" s="7" t="inlineStr">
+        <is>
+          <t>Try overriding without a reason; then sign in as HR Specialist and look for the Override button.</t>
+        </is>
+      </c>
+      <c r="E44" s="7" t="inlineStr">
+        <is>
+          <t>No reason → rejected (reason is required). HR Specialist doesn't see the Override button (HR Admin only).</t>
+        </is>
+      </c>
+      <c r="F44" s="8" t="inlineStr"/>
+      <c r="G44" s="7" t="inlineStr"/>
+    </row>
+    <row r="45" ht="42" customHeight="1">
+      <c r="A45" s="9" t="inlineStr">
+        <is>
+          <t>SEC-B1</t>
+        </is>
+      </c>
+      <c r="B45" s="10" t="inlineStr">
+        <is>
+          <t>Permissions (Phase B)</t>
+        </is>
+      </c>
+      <c r="C45" s="10" t="inlineStr">
+        <is>
+          <t>Employee</t>
+        </is>
+      </c>
+      <c r="D45" s="10" t="inlineStr">
+        <is>
+          <t>Sign in as an Employee. Open another employee's review URL directly (/performance/reviews/&lt;id&gt;).</t>
+        </is>
+      </c>
+      <c r="E45" s="10" t="inlineStr">
+        <is>
+          <t>The competency and scoring data of another employee is NOT accessible (hierarchy guard — access denied / error).</t>
+        </is>
+      </c>
+      <c r="F45" s="8" t="inlineStr"/>
+      <c r="G45" s="10" t="inlineStr"/>
+    </row>
   </sheetData>
   <dataValidations count="1">
-    <dataValidation sqref="F2:F30" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="F2:F45" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"Pass,Fail,Blocked,Not Run"</formula1>
     </dataValidation>
   </dataValidations>
@@ -1542,7 +1977,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="B1:E14"/>
+  <dimension ref="B1:E17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="3" customWidth="1" min="1" max="1"/>
@@ -1624,30 +2059,60 @@
     <row r="8">
       <c r="B8" s="13" t="inlineStr">
         <is>
-          <t>Permissions (SEC)</t>
+          <t>Goal-plan approval + progress trail (GPL/GPT)</t>
         </is>
       </c>
       <c r="C8" s="14" t="n"/>
       <c r="D8" s="15" t="n"/>
       <c r="E8" s="15" t="n"/>
     </row>
+    <row r="9">
+      <c r="B9" s="13" t="inlineStr">
+        <is>
+          <t>Competency assessment (CMP)</t>
+        </is>
+      </c>
+      <c r="C9" s="14" t="n"/>
+      <c r="D9" s="15" t="n"/>
+      <c r="E9" s="15" t="n"/>
+    </row>
+    <row r="10">
+      <c r="B10" s="13" t="inlineStr">
+        <is>
+          <t>Weighted scoring + override (SCR/OVR)</t>
+        </is>
+      </c>
+      <c r="C10" s="14" t="n"/>
+      <c r="D10" s="15" t="n"/>
+      <c r="E10" s="15" t="n"/>
+    </row>
     <row r="11">
-      <c r="B11" s="16" t="inlineStr">
+      <c r="B11" s="13" t="inlineStr">
+        <is>
+          <t>Permissions (SEC)</t>
+        </is>
+      </c>
+      <c r="C11" s="14" t="n"/>
+      <c r="D11" s="15" t="n"/>
+      <c r="E11" s="15" t="n"/>
+    </row>
+    <row r="14">
+      <c r="B14" s="16" t="inlineStr">
         <is>
           <t>Overall decision (SHIP / DON'T SHIP):</t>
         </is>
       </c>
-      <c r="C11" s="14" t="n"/>
-    </row>
-    <row r="13">
-      <c r="B13" s="17" t="inlineStr">
+      <c r="C14" s="14" t="n"/>
+    </row>
+    <row r="16">
+      <c r="B16" s="17" t="inlineStr">
         <is>
           <t>Tester name:</t>
         </is>
       </c>
     </row>
-    <row r="14">
-      <c r="B14" s="17" t="inlineStr">
+    <row r="17">
+      <c r="B17" s="17" t="inlineStr">
         <is>
           <t>Date:</t>
         </is>
@@ -1655,7 +2120,7 @@
     </row>
   </sheetData>
   <dataValidations count="1">
-    <dataValidation sqref="C4 C5 C6 C7 C8" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="C4 C5 C6 C7 C8 C9 C10 C11" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"Pass,Fail,Blocked,Not Run"</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>

<commit_message>
docs(performance): HCM_12 UAT grown to Phase D — 60 cases (360/appeals/committee)
Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/PRD/HCM_12_Performance_Management_Multi_Tenant_PRD/Performance_UAT_Test_Script.xlsx
+++ b/PRD/HCM_12_Performance_Management_Multi_Tenant_PRD/Performance_UAT_Test_Script.xlsx
@@ -585,7 +585,7 @@
       </c>
       <c r="C7" s="4" t="inlineStr">
         <is>
-          <t>Phase A (configuration foundation): rating scales with score bands (M388), review templates with weighted sections + cycle audience scoping (M389), KPI library + per-cycle assignments with automatic achievement/rating scoring (M390), OKR objectives + key results + check-ins with progress roll-up (M391). Phase B (goals &amp; scoring): goal-plan approval workflow Employee→Manager with weights-must-total-100 validation + progress-update audit trail (M392), per-review competency assessment with position-requirement seeding and gap analysis (M393), §18 weighted section scoring + score→band conversion + HR rating override with preserved original (M394).</t>
+          <t>Phase A: rating scales (M388), review templates + cycle scoping (M389), KPI library + auto-scored assignments (M390), OKR + check-ins (M391). Phase B: goal-plan approval workflow + progress trail (M392), competency assessment with gap analysis (M393), §18 weighted scoring + band conversion + HR override (M394). Phase C: 360° reviewer nominations + questionnaires + min/max rules (M395). Phase D: result acknowledgement + appeals with preserved original rating (M396), calibration committee access control + HR-only calibration notes + outlier/leniency view (M397).</t>
         </is>
       </c>
     </row>
@@ -636,7 +636,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G45"/>
+  <dimension ref="A1:G60"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -1961,9 +1961,444 @@
       <c r="F45" s="8" t="inlineStr"/>
       <c r="G45" s="10" t="inlineStr"/>
     </row>
+    <row r="46" ht="72" customHeight="1">
+      <c r="A46" s="6" t="inlineStr">
+        <is>
+          <t>Q36-01</t>
+        </is>
+      </c>
+      <c r="B46" s="7" t="inlineStr">
+        <is>
+          <t>Questionnaires (M395)</t>
+        </is>
+      </c>
+      <c r="C46" s="7" t="inlineStr">
+        <is>
+          <t>HR Admin</t>
+        </is>
+      </c>
+      <c r="D46" s="7" t="inlineStr">
+        <is>
+          <t>Performance → 360° nominations → Questionnaires tab → 'New questionnaire'. Code=STD_360, Name='Standard 360'. Add 3 questions: a RATING/COMPETENCY, a RATING/LEADERSHIP and a TEXT/IMPROVEMENT one. Save.</t>
+        </is>
+      </c>
+      <c r="E46" s="7" t="inlineStr">
+        <is>
+          <t>The questionnaire appears with 3 questions (expand the row to see types/categories/required tags).</t>
+        </is>
+      </c>
+      <c r="F46" s="8" t="inlineStr"/>
+      <c r="G46" s="7" t="inlineStr"/>
+    </row>
+    <row r="47" ht="57" customHeight="1">
+      <c r="A47" s="9" t="inlineStr">
+        <is>
+          <t>N36-01</t>
+        </is>
+      </c>
+      <c r="B47" s="10" t="inlineStr">
+        <is>
+          <t>Nomination (M395)</t>
+        </is>
+      </c>
+      <c r="C47" s="10" t="inlineStr">
+        <is>
+          <t>HR Admin</t>
+        </is>
+      </c>
+      <c r="D47" s="10" t="inlineStr">
+        <is>
+          <t>Nominations tab → pick a cycle → 'Nominate reviewer'. Subject=employee A, Reviewer=employee B, Relationship=PEER, Questionnaire=STD_360, Anonymous ON. Nominate.</t>
+        </is>
+      </c>
+      <c r="E47" s="10" t="inlineStr">
+        <is>
+          <t>A NOMINATED row appears with the PEER tag, questionnaire name and 'anonymous' tag.</t>
+        </is>
+      </c>
+      <c r="F47" s="8" t="inlineStr"/>
+      <c r="G47" s="10" t="inlineStr"/>
+    </row>
+    <row r="48" ht="42" customHeight="1">
+      <c r="A48" s="6" t="inlineStr">
+        <is>
+          <t>N36-02</t>
+        </is>
+      </c>
+      <c r="B48" s="7" t="inlineStr">
+        <is>
+          <t>Duplicate guard (M395)</t>
+        </is>
+      </c>
+      <c r="C48" s="7" t="inlineStr">
+        <is>
+          <t>HR Admin</t>
+        </is>
+      </c>
+      <c r="D48" s="7" t="inlineStr">
+        <is>
+          <t>Nominate the SAME reviewer for the SAME subject in the SAME cycle again.</t>
+        </is>
+      </c>
+      <c r="E48" s="7" t="inlineStr">
+        <is>
+          <t>Rejected — this reviewer is already nominated for the subject in this cycle.</t>
+        </is>
+      </c>
+      <c r="F48" s="8" t="inlineStr"/>
+      <c r="G48" s="7" t="inlineStr"/>
+    </row>
+    <row r="49" ht="72" customHeight="1">
+      <c r="A49" s="9" t="inlineStr">
+        <is>
+          <t>N36-03</t>
+        </is>
+      </c>
+      <c r="B49" s="10" t="inlineStr">
+        <is>
+          <t>Approve + respond (M395)</t>
+        </is>
+      </c>
+      <c r="C49" s="10" t="inlineStr">
+        <is>
+          <t>HR Admin</t>
+        </is>
+      </c>
+      <c r="D49" s="10" t="inlineStr">
+        <is>
+          <t>On the NOMINATED row click Approve, then Respond. The STD_360 questions render (stars for RATING, text area for TEXT). Answer required questions, set Overall rating 4, strengths/improvements. Submit.</t>
+        </is>
+      </c>
+      <c r="E49" s="10" t="inlineStr">
+        <is>
+          <t>Status becomes COMPLETED. Performance → Feedback shows a new ANONYMOUS PEER feedback for subject A (answers stored under competencies).</t>
+        </is>
+      </c>
+      <c r="F49" s="8" t="inlineStr"/>
+      <c r="G49" s="10" t="inlineStr"/>
+    </row>
+    <row r="50" ht="30" customHeight="1">
+      <c r="A50" s="6" t="inlineStr">
+        <is>
+          <t>N36-04</t>
+        </is>
+      </c>
+      <c r="B50" s="7" t="inlineStr">
+        <is>
+          <t>Decline (M395)</t>
+        </is>
+      </c>
+      <c r="C50" s="7" t="inlineStr">
+        <is>
+          <t>HR Admin</t>
+        </is>
+      </c>
+      <c r="D50" s="7" t="inlineStr">
+        <is>
+          <t>Nominate another reviewer, then Decline with a reason.</t>
+        </is>
+      </c>
+      <c r="E50" s="7" t="inlineStr">
+        <is>
+          <t>Status becomes DECLINED and the reason shows on the row.</t>
+        </is>
+      </c>
+      <c r="F50" s="8" t="inlineStr"/>
+      <c r="G50" s="7" t="inlineStr"/>
+    </row>
+    <row r="51" ht="57" customHeight="1">
+      <c r="A51" s="9" t="inlineStr">
+        <is>
+          <t>N36-05</t>
+        </is>
+      </c>
+      <c r="B51" s="10" t="inlineStr">
+        <is>
+          <t>Min/max rules (M395)</t>
+        </is>
+      </c>
+      <c r="C51" s="10" t="inlineStr">
+        <is>
+          <t>HR Admin</t>
+        </is>
+      </c>
+      <c r="D51" s="10" t="inlineStr">
+        <is>
+          <t>Edit the review cycle: set Max reviewers=2 and Min reviewers=2 (cycle form). Then try nominating a 3rd live reviewer for the same subject.</t>
+        </is>
+      </c>
+      <c r="E51" s="10" t="inlineStr">
+        <is>
+          <t>Rejected — maximum reviewers reached. The summary tags next to the filters show 'completed / min' in red until 2 responses are completed.</t>
+        </is>
+      </c>
+      <c r="F51" s="8" t="inlineStr"/>
+      <c r="G51" s="10" t="inlineStr"/>
+    </row>
+    <row r="52" ht="57" customHeight="1">
+      <c r="A52" s="6" t="inlineStr">
+        <is>
+          <t>ACK-01</t>
+        </is>
+      </c>
+      <c r="B52" s="7" t="inlineStr">
+        <is>
+          <t>Acknowledgement (M396)</t>
+        </is>
+      </c>
+      <c r="C52" s="7" t="inlineStr">
+        <is>
+          <t>HR Admin</t>
+        </is>
+      </c>
+      <c r="D52" s="7" t="inlineStr">
+        <is>
+          <t>Open a review that HAS a final rating. In 'Acknowledgement &amp; appeals' click 'Acknowledge result' with a comment, dispute OFF.</t>
+        </is>
+      </c>
+      <c r="E52" s="7" t="inlineStr">
+        <is>
+          <t>The card shows 'Acknowledged &lt;time&gt;' with a green 'accepted' tag; the Acknowledge button disappears (one-shot).</t>
+        </is>
+      </c>
+      <c r="F52" s="8" t="inlineStr"/>
+      <c r="G52" s="7" t="inlineStr"/>
+    </row>
+    <row r="53" ht="42" customHeight="1">
+      <c r="A53" s="9" t="inlineStr">
+        <is>
+          <t>ACK-02</t>
+        </is>
+      </c>
+      <c r="B53" s="10" t="inlineStr">
+        <is>
+          <t>Ack guards (M396)</t>
+        </is>
+      </c>
+      <c r="C53" s="10" t="inlineStr">
+        <is>
+          <t>HR Admin</t>
+        </is>
+      </c>
+      <c r="D53" s="10" t="inlineStr">
+        <is>
+          <t>Try acknowledging the same review again (or a review with NO final rating).</t>
+        </is>
+      </c>
+      <c r="E53" s="10" t="inlineStr">
+        <is>
+          <t>Already acknowledged → rejected; no final rating → the button is not offered / rejected.</t>
+        </is>
+      </c>
+      <c r="F53" s="8" t="inlineStr"/>
+      <c r="G53" s="10" t="inlineStr"/>
+    </row>
+    <row r="54" ht="72" customHeight="1">
+      <c r="A54" s="6" t="inlineStr">
+        <is>
+          <t>APL-01</t>
+        </is>
+      </c>
+      <c r="B54" s="7" t="inlineStr">
+        <is>
+          <t>Appeal happy path (M396)</t>
+        </is>
+      </c>
+      <c r="C54" s="7" t="inlineStr">
+        <is>
+          <t>HR Admin</t>
+        </is>
+      </c>
+      <c r="D54" s="7" t="inlineStr">
+        <is>
+          <t>On a review with a final rating click 'Submit appeal' with a reason. Then (as HR) 'Take under review' → 'Decide' → APPROVED with Adjusted rating 4.2 and notes.</t>
+        </is>
+      </c>
+      <c r="E54" s="7" t="inlineStr">
+        <is>
+          <t>Appeal goes SUBMITTED → UNDER_REVIEW → APPROVED. The review's final rating becomes 4.20 with the 'overridden' tag and the ORIGINAL rating preserved in the Weighted-scores card (§37.12). Close the appeal → CLOSED.</t>
+        </is>
+      </c>
+      <c r="F54" s="8" t="inlineStr"/>
+      <c r="G54" s="7" t="inlineStr"/>
+    </row>
+    <row r="55" ht="57" customHeight="1">
+      <c r="A55" s="9" t="inlineStr">
+        <is>
+          <t>APL-02</t>
+        </is>
+      </c>
+      <c r="B55" s="10" t="inlineStr">
+        <is>
+          <t>Appeal reject/return (M396)</t>
+        </is>
+      </c>
+      <c r="C55" s="10" t="inlineStr">
+        <is>
+          <t>HR Admin</t>
+        </is>
+      </c>
+      <c r="D55" s="10" t="inlineStr">
+        <is>
+          <t>Submit an appeal on another review; decide REJECTED (rating unchanged). Submit a third; decide RETURNED, then click Resubmit.</t>
+        </is>
+      </c>
+      <c r="E55" s="10" t="inlineStr">
+        <is>
+          <t>REJECTED keeps the rating; RETURNED lets the employee resubmit (status back to SUBMITTED). Only ONE live appeal per review is allowed.</t>
+        </is>
+      </c>
+      <c r="F55" s="8" t="inlineStr"/>
+      <c r="G55" s="10" t="inlineStr"/>
+    </row>
+    <row r="56" ht="57" customHeight="1">
+      <c r="A56" s="6" t="inlineStr">
+        <is>
+          <t>COM-01</t>
+        </is>
+      </c>
+      <c r="B56" s="7" t="inlineStr">
+        <is>
+          <t>Committee (M397)</t>
+        </is>
+      </c>
+      <c r="C56" s="7" t="inlineStr">
+        <is>
+          <t>HR Admin</t>
+        </is>
+      </c>
+      <c r="D56" s="7" t="inlineStr">
+        <is>
+          <t>Performance → Review cycles → open a cycle's Calibration page. On a session click 'Committee'. Add a manager as MEMBER and someone as OBSERVER.</t>
+        </is>
+      </c>
+      <c r="E56" s="7" t="inlineStr">
+        <is>
+          <t>Both appear with role tags. (CHAIR/MEMBER may calibrate; OBSERVER is read-only.)</t>
+        </is>
+      </c>
+      <c r="F56" s="8" t="inlineStr"/>
+      <c r="G56" s="7" t="inlineStr"/>
+    </row>
+    <row r="57" ht="42" customHeight="1">
+      <c r="A57" s="9" t="inlineStr">
+        <is>
+          <t>COM-02</t>
+        </is>
+      </c>
+      <c r="B57" s="10" t="inlineStr">
+        <is>
+          <t>Committee gate (M397)</t>
+        </is>
+      </c>
+      <c r="C57" s="10" t="inlineStr">
+        <is>
+          <t>Manager</t>
+        </is>
+      </c>
+      <c r="D57" s="10" t="inlineStr">
+        <is>
+          <t>Sign in as a manager NOT on any committee and open the calibration board URL for the cycle.</t>
+        </is>
+      </c>
+      <c r="E57" s="10" t="inlineStr">
+        <is>
+          <t>Access denied — the board requires committee membership for managers (HR roles always may).</t>
+        </is>
+      </c>
+      <c r="F57" s="8" t="inlineStr"/>
+      <c r="G57" s="10" t="inlineStr"/>
+    </row>
+    <row r="58" ht="57" customHeight="1">
+      <c r="A58" s="6" t="inlineStr">
+        <is>
+          <t>COM-03</t>
+        </is>
+      </c>
+      <c r="B58" s="7" t="inlineStr">
+        <is>
+          <t>Committee calibrate (M397)</t>
+        </is>
+      </c>
+      <c r="C58" s="7" t="inlineStr">
+        <is>
+          <t>Manager</t>
+        </is>
+      </c>
+      <c r="D58" s="7" t="inlineStr">
+        <is>
+          <t>Add the manager to the committee as MEMBER (as HR), start the session, then as that manager calibrate a review on the board.</t>
+        </is>
+      </c>
+      <c r="E58" s="7" t="inlineStr">
+        <is>
+          <t>The calibrate saves — committee MEMBERs may calibrate while the session is IN_PROGRESS.</t>
+        </is>
+      </c>
+      <c r="F58" s="8" t="inlineStr"/>
+      <c r="G58" s="7" t="inlineStr"/>
+    </row>
+    <row r="59" ht="57" customHeight="1">
+      <c r="A59" s="9" t="inlineStr">
+        <is>
+          <t>VIS-01</t>
+        </is>
+      </c>
+      <c r="B59" s="10" t="inlineStr">
+        <is>
+          <t>Notes visibility (M397)</t>
+        </is>
+      </c>
+      <c r="C59" s="10" t="inlineStr">
+        <is>
+          <t>Employee</t>
+        </is>
+      </c>
+      <c r="D59" s="10" t="inlineStr">
+        <is>
+          <t>As an employee whose review has calibration notes, open your own review.</t>
+        </is>
+      </c>
+      <c r="E59" s="10" t="inlineStr">
+        <is>
+          <t>Calibration notes (and any override reason) are NOT visible to you — they are HR/committee-only (§19.3). Signing in as HR shows them.</t>
+        </is>
+      </c>
+      <c r="F59" s="8" t="inlineStr"/>
+      <c r="G59" s="10" t="inlineStr"/>
+    </row>
+    <row r="60" ht="57" customHeight="1">
+      <c r="A60" s="6" t="inlineStr">
+        <is>
+          <t>OUT-01</t>
+        </is>
+      </c>
+      <c r="B60" s="7" t="inlineStr">
+        <is>
+          <t>Outliers (M397)</t>
+        </is>
+      </c>
+      <c r="C60" s="7" t="inlineStr">
+        <is>
+          <t>HR Admin</t>
+        </is>
+      </c>
+      <c r="D60" s="7" t="inlineStr">
+        <is>
+          <t>On the Calibration page scroll to 'Outliers &amp; manager leniency'.</t>
+        </is>
+      </c>
+      <c r="E60" s="7" t="inlineStr">
+        <is>
+          <t>Shows the cycle average, a per-manager average with Δ tags (orange/red when ≥0.5 off), and individual reviews ≥1.0 from the cycle average.</t>
+        </is>
+      </c>
+      <c r="F60" s="8" t="inlineStr"/>
+      <c r="G60" s="7" t="inlineStr"/>
+    </row>
   </sheetData>
   <dataValidations count="1">
-    <dataValidation sqref="F2:F45" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="F2:F60" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"Pass,Fail,Blocked,Not Run"</formula1>
     </dataValidation>
   </dataValidations>
@@ -1977,7 +2412,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="B1:E17"/>
+  <dimension ref="B1:E20"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="3" customWidth="1" min="1" max="1"/>
@@ -2089,30 +2524,60 @@
     <row r="11">
       <c r="B11" s="13" t="inlineStr">
         <is>
-          <t>Permissions (SEC)</t>
+          <t>360° nominations + questionnaires (Q36/N36)</t>
         </is>
       </c>
       <c r="C11" s="14" t="n"/>
       <c r="D11" s="15" t="n"/>
       <c r="E11" s="15" t="n"/>
     </row>
+    <row r="12">
+      <c r="B12" s="13" t="inlineStr">
+        <is>
+          <t>Acknowledgement + appeals (ACK/APL)</t>
+        </is>
+      </c>
+      <c r="C12" s="14" t="n"/>
+      <c r="D12" s="15" t="n"/>
+      <c r="E12" s="15" t="n"/>
+    </row>
+    <row r="13">
+      <c r="B13" s="13" t="inlineStr">
+        <is>
+          <t>Calibration committee + outliers (COM/VIS/OUT)</t>
+        </is>
+      </c>
+      <c r="C13" s="14" t="n"/>
+      <c r="D13" s="15" t="n"/>
+      <c r="E13" s="15" t="n"/>
+    </row>
     <row r="14">
-      <c r="B14" s="16" t="inlineStr">
+      <c r="B14" s="13" t="inlineStr">
+        <is>
+          <t>Permissions (SEC)</t>
+        </is>
+      </c>
+      <c r="C14" s="14" t="n"/>
+      <c r="D14" s="15" t="n"/>
+      <c r="E14" s="15" t="n"/>
+    </row>
+    <row r="17">
+      <c r="B17" s="16" t="inlineStr">
         <is>
           <t>Overall decision (SHIP / DON'T SHIP):</t>
         </is>
       </c>
-      <c r="C14" s="14" t="n"/>
-    </row>
-    <row r="16">
-      <c r="B16" s="17" t="inlineStr">
+      <c r="C17" s="14" t="n"/>
+    </row>
+    <row r="19">
+      <c r="B19" s="17" t="inlineStr">
         <is>
           <t>Tester name:</t>
         </is>
       </c>
     </row>
-    <row r="17">
-      <c r="B17" s="17" t="inlineStr">
+    <row r="20">
+      <c r="B20" s="17" t="inlineStr">
         <is>
           <t>Date:</t>
         </is>
@@ -2120,7 +2585,7 @@
     </row>
   </sheetData>
   <dataValidations count="1">
-    <dataValidation sqref="C4 C5 C6 C7 C8 C9 C10 C11" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="C4 C5 C6 C7 C8 C9 C10 C11 C12 C13 C14" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"Pass,Fail,Blocked,Not Run"</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>

<commit_message>
docs(performance): HCM_12 UAT complete A–F — 73 cases
Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/PRD/HCM_12_Performance_Management_Multi_Tenant_PRD/Performance_UAT_Test_Script.xlsx
+++ b/PRD/HCM_12_Performance_Management_Multi_Tenant_PRD/Performance_UAT_Test_Script.xlsx
@@ -585,7 +585,7 @@
       </c>
       <c r="C7" s="4" t="inlineStr">
         <is>
-          <t>Phase A: rating scales (M388), review templates + cycle scoping (M389), KPI library + auto-scored assignments (M390), OKR + check-ins (M391). Phase B: goal-plan approval workflow + progress trail (M392), competency assessment with gap analysis (M393), §18 weighted scoring + band conversion + HR override (M394). Phase C: 360° reviewer nominations + questionnaires + min/max rules (M395). Phase D: result acknowledgement + appeals with preserved original rating (M396), calibration committee access control + HR-only calibration notes + outlier/leniency view (M397).</t>
+          <t>ALL PHASES A–F COMPLETE. A: rating scales (M388), review templates + cycle scoping (M389), KPI library + auto-scored assignments (M390), OKR + check-ins (M391). B: goal-plan approval workflow + progress trail (M392), competency assessment with gaps (M393), §18 weighted scoring + band + HR override (M394). C: 360° nominations + questionnaires + min/max rules (M395). D: acknowledgement + appeals (M396), calibration committee + HR-only notes + outliers (M397). E: PIPs (M398), development plans (M399), continuous feedback + check-ins (M400). F: HR dashboard (M401), notifications + comp-bridge finalised-only guard (M402).</t>
         </is>
       </c>
     </row>
@@ -636,7 +636,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G60"/>
+  <dimension ref="A1:G73"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -2396,9 +2396,386 @@
       <c r="F60" s="8" t="inlineStr"/>
       <c r="G60" s="7" t="inlineStr"/>
     </row>
+    <row r="61" ht="57" customHeight="1">
+      <c r="A61" s="9" t="inlineStr">
+        <is>
+          <t>PIP-01</t>
+        </is>
+      </c>
+      <c r="B61" s="10" t="inlineStr">
+        <is>
+          <t>PIP create (M398)</t>
+        </is>
+      </c>
+      <c r="C61" s="10" t="inlineStr">
+        <is>
+          <t>HR Admin</t>
+        </is>
+      </c>
+      <c r="D61" s="10" t="inlineStr">
+        <is>
+          <t>Performance → PIPs → 'New PIP'. Pick an employee, reason, start today, end +60 days, objectives + success criteria. Save.</t>
+        </is>
+      </c>
+      <c r="E61" s="10" t="inlineStr">
+        <is>
+          <t>A DRAFT PIP appears. Trying to create a SECOND PIP for the same employee is rejected (one live PIP per employee).</t>
+        </is>
+      </c>
+      <c r="F61" s="8" t="inlineStr"/>
+      <c r="G61" s="10" t="inlineStr"/>
+    </row>
+    <row r="62" ht="57" customHeight="1">
+      <c r="A62" s="6" t="inlineStr">
+        <is>
+          <t>PIP-02</t>
+        </is>
+      </c>
+      <c r="B62" s="7" t="inlineStr">
+        <is>
+          <t>PIP lifecycle (M398)</t>
+        </is>
+      </c>
+      <c r="C62" s="7" t="inlineStr">
+        <is>
+          <t>HR Admin</t>
+        </is>
+      </c>
+      <c r="D62" s="7" t="inlineStr">
+        <is>
+          <t>Open the PIP → Activate. Then 'Acknowledge (employee)' with a comment. Then record a checkpoint (rating 2, comment).</t>
+        </is>
+      </c>
+      <c r="E62" s="7" t="inlineStr">
+        <is>
+          <t>DRAFT → ACTIVE (employee is notified) → ACKNOWLEDGED → after the checkpoint IN_PROGRESS. Checkpoints are blocked until acknowledged; the timeline shows the 2/5 rating in red.</t>
+        </is>
+      </c>
+      <c r="F62" s="8" t="inlineStr"/>
+      <c r="G62" s="7" t="inlineStr"/>
+    </row>
+    <row r="63" ht="57" customHeight="1">
+      <c r="A63" s="9" t="inlineStr">
+        <is>
+          <t>PIP-03</t>
+        </is>
+      </c>
+      <c r="B63" s="10" t="inlineStr">
+        <is>
+          <t>PIP extend + close (M398)</t>
+        </is>
+      </c>
+      <c r="C63" s="10" t="inlineStr">
+        <is>
+          <t>HR Admin</t>
+        </is>
+      </c>
+      <c r="D63" s="10" t="inlineStr">
+        <is>
+          <t>Extend the PIP with a later end date; then 'Close with outcome' = IMPROVED with notes.</t>
+        </is>
+      </c>
+      <c r="E63" s="10" t="inlineStr">
+        <is>
+          <t>EXTENDED shows the new window; closing with IMPROVED → COMPLETED_SUCCESS (any other outcome → FAILED). Outcome decisions are HR-only; history stays (nothing is deleted).</t>
+        </is>
+      </c>
+      <c r="F63" s="8" t="inlineStr"/>
+      <c r="G63" s="10" t="inlineStr"/>
+    </row>
+    <row r="64" ht="42" customHeight="1">
+      <c r="A64" s="6" t="inlineStr">
+        <is>
+          <t>PIP-04</t>
+        </is>
+      </c>
+      <c r="B64" s="7" t="inlineStr">
+        <is>
+          <t>PIP evidence (M398)</t>
+        </is>
+      </c>
+      <c r="C64" s="7" t="inlineStr">
+        <is>
+          <t>HR Admin</t>
+        </is>
+      </c>
+      <c r="D64" s="7" t="inlineStr">
+        <is>
+          <t>In the PIP drawer upload a file under 'Evidence / documents'.</t>
+        </is>
+      </c>
+      <c r="E64" s="7" t="inlineStr">
+        <is>
+          <t>The file attaches via the standard uploader (M16 registry) and reloads with the PIP.</t>
+        </is>
+      </c>
+      <c r="F64" s="8" t="inlineStr"/>
+      <c r="G64" s="7" t="inlineStr"/>
+    </row>
+    <row r="65" ht="57" customHeight="1">
+      <c r="A65" s="9" t="inlineStr">
+        <is>
+          <t>DVP-01</t>
+        </is>
+      </c>
+      <c r="B65" s="10" t="inlineStr">
+        <is>
+          <t>Dev plan (M399)</t>
+        </is>
+      </c>
+      <c r="C65" s="10" t="inlineStr">
+        <is>
+          <t>HR Admin</t>
+        </is>
+      </c>
+      <c r="D65" s="10" t="inlineStr">
+        <is>
+          <t>Performance → Development plans → 'New plan'. Employee, title, 3 actions of different types (e.g. Training course / Coaching / Stretch assignment). Save.</t>
+        </is>
+      </c>
+      <c r="E65" s="10" t="inlineStr">
+        <is>
+          <t>The plan appears at 0%; expanding shows the 3 typed actions.</t>
+        </is>
+      </c>
+      <c r="F65" s="8" t="inlineStr"/>
+      <c r="G65" s="10" t="inlineStr"/>
+    </row>
+    <row r="66" ht="42" customHeight="1">
+      <c r="A66" s="6" t="inlineStr">
+        <is>
+          <t>DVP-02</t>
+        </is>
+      </c>
+      <c r="B66" s="7" t="inlineStr">
+        <is>
+          <t>Dev plan progress (M399)</t>
+        </is>
+      </c>
+      <c r="C66" s="7" t="inlineStr">
+        <is>
+          <t>HR Admin</t>
+        </is>
+      </c>
+      <c r="D66" s="7" t="inlineStr">
+        <is>
+          <t>Mark one action Done, one In progress.</t>
+        </is>
+      </c>
+      <c r="E66" s="7" t="inlineStr">
+        <is>
+          <t>Progress becomes 33.33% and status flips to IN PROGRESS. Marking ALL actions Done → 100% and the plan auto-COMPLETES.</t>
+        </is>
+      </c>
+      <c r="F66" s="8" t="inlineStr"/>
+      <c r="G66" s="7" t="inlineStr"/>
+    </row>
+    <row r="67" ht="57" customHeight="1">
+      <c r="A67" s="9" t="inlineStr">
+        <is>
+          <t>DVP-03</t>
+        </is>
+      </c>
+      <c r="B67" s="10" t="inlineStr">
+        <is>
+          <t>From-gaps plan (M399)</t>
+        </is>
+      </c>
+      <c r="C67" s="10" t="inlineStr">
+        <is>
+          <t>HR Admin</t>
+        </is>
+      </c>
+      <c r="D67" s="10" t="inlineStr">
+        <is>
+          <t>On a review with positive competency gaps call the from-review generation (POST /api/performance/dev-plans/from-review/&lt;reviewId&gt; — or verify via the API tool).</t>
+        </is>
+      </c>
+      <c r="E67" s="10" t="inlineStr">
+        <is>
+          <t>A plan 'Close competency gaps — review …' is created with one TRAINING_COURSE action per positive gap (§21.3).</t>
+        </is>
+      </c>
+      <c r="F67" s="8" t="inlineStr"/>
+      <c r="G67" s="10" t="inlineStr"/>
+    </row>
+    <row r="68" ht="57" customHeight="1">
+      <c r="A68" s="6" t="inlineStr">
+        <is>
+          <t>CFB-01</t>
+        </is>
+      </c>
+      <c r="B68" s="7" t="inlineStr">
+        <is>
+          <t>Feedback (M400)</t>
+        </is>
+      </c>
+      <c r="C68" s="7" t="inlineStr">
+        <is>
+          <t>HR Admin</t>
+        </is>
+      </c>
+      <c r="D68" s="7" t="inlineStr">
+        <is>
+          <t>Performance → Check-ins → pick an employee → 'Give feedback': PRAISE, employee-visible, tags 'teamwork'. Then a second one: kind NOTE, visibility 'Private manager note'.</t>
+        </is>
+      </c>
+      <c r="E68" s="7" t="inlineStr">
+        <is>
+          <t>Both appear in the Feedback timeline; the private one carries a red 'manager-private' tag.</t>
+        </is>
+      </c>
+      <c r="F68" s="8" t="inlineStr"/>
+      <c r="G68" s="7" t="inlineStr"/>
+    </row>
+    <row r="69" ht="42" customHeight="1">
+      <c r="A69" s="9" t="inlineStr">
+        <is>
+          <t>CFB-02</t>
+        </is>
+      </c>
+      <c r="B69" s="10" t="inlineStr">
+        <is>
+          <t>Private-note visibility (M400)</t>
+        </is>
+      </c>
+      <c r="C69" s="10" t="inlineStr">
+        <is>
+          <t>Employee</t>
+        </is>
+      </c>
+      <c r="D69" s="10" t="inlineStr">
+        <is>
+          <t>Sign in as that employee and load your feedback (via My Workspace/API).</t>
+        </is>
+      </c>
+      <c r="E69" s="10" t="inlineStr">
+        <is>
+          <t>The PRAISE note is visible; the MANAGER_PRIVATE note is NOT returned to the employee (§22.1).</t>
+        </is>
+      </c>
+      <c r="F69" s="8" t="inlineStr"/>
+      <c r="G69" s="10" t="inlineStr"/>
+    </row>
+    <row r="70" ht="57" customHeight="1">
+      <c r="A70" s="6" t="inlineStr">
+        <is>
+          <t>CIN-01</t>
+        </is>
+      </c>
+      <c r="B70" s="7" t="inlineStr">
+        <is>
+          <t>Check-in (M400)</t>
+        </is>
+      </c>
+      <c r="C70" s="7" t="inlineStr">
+        <is>
+          <t>HR Admin</t>
+        </is>
+      </c>
+      <c r="D70" s="7" t="inlineStr">
+        <is>
+          <t>'Record check-in': today, One-to-one, discussion notes + action items + follow-up date. Save. Then click Acknowledge on the row.</t>
+        </is>
+      </c>
+      <c r="E70" s="7" t="inlineStr">
+        <is>
+          <t>The check-in row appears with notes/actions/follow-up; acknowledging turns the Ack column into a green 'acknowledged' tag (one-shot).</t>
+        </is>
+      </c>
+      <c r="F70" s="8" t="inlineStr"/>
+      <c r="G70" s="7" t="inlineStr"/>
+    </row>
+    <row r="71" ht="72" customHeight="1">
+      <c r="A71" s="9" t="inlineStr">
+        <is>
+          <t>DSH-01</t>
+        </is>
+      </c>
+      <c r="B71" s="10" t="inlineStr">
+        <is>
+          <t>Dashboard (M401)</t>
+        </is>
+      </c>
+      <c r="C71" s="10" t="inlineStr">
+        <is>
+          <t>HR Admin</t>
+        </is>
+      </c>
+      <c r="D71" s="10" t="inlineStr">
+        <is>
+          <t>Performance → Dashboard → pick the test cycle.</t>
+        </is>
+      </c>
+      <c r="E71" s="10" t="inlineStr">
+        <is>
+          <t>Stat cards populate (reviews, pending acknowledgement, disputed, goal plans awaiting approval, open appeals, active PIPs, active dev plans) plus the status funnel, rating distribution and top/bottom-5 performers.</t>
+        </is>
+      </c>
+      <c r="F71" s="8" t="inlineStr"/>
+      <c r="G71" s="10" t="inlineStr"/>
+    </row>
+    <row r="72" ht="57" customHeight="1">
+      <c r="A72" s="6" t="inlineStr">
+        <is>
+          <t>NTF-01</t>
+        </is>
+      </c>
+      <c r="B72" s="7" t="inlineStr">
+        <is>
+          <t>Notifications (M402)</t>
+        </is>
+      </c>
+      <c r="C72" s="7" t="inlineStr">
+        <is>
+          <t>Employee</t>
+        </is>
+      </c>
+      <c r="D72" s="7" t="inlineStr">
+        <is>
+          <t>After a manager approves/rejects your goal plan, HR decides your appeal, or a PIP is activated for you — check the notifications bell.</t>
+        </is>
+      </c>
+      <c r="E72" s="7" t="inlineStr">
+        <is>
+          <t>In-app notifications arrive for each event (goal plan approved/rejected, appeal decision incl. adjusted rating, PIP activated).</t>
+        </is>
+      </c>
+      <c r="F72" s="8" t="inlineStr"/>
+      <c r="G72" s="7" t="inlineStr"/>
+    </row>
+    <row r="73" ht="57" customHeight="1">
+      <c r="A73" s="9" t="inlineStr">
+        <is>
+          <t>CMP-G1</t>
+        </is>
+      </c>
+      <c r="B73" s="10" t="inlineStr">
+        <is>
+          <t>Comp-bridge guard (M402)</t>
+        </is>
+      </c>
+      <c r="C73" s="10" t="inlineStr">
+        <is>
+          <t>HR Admin</t>
+        </is>
+      </c>
+      <c r="D73" s="10" t="inlineStr">
+        <is>
+          <t>Create a bonus run (Comp &amp; Benefits → Bonus runs) for a cycle where one review is APPROVED/COMPLETED and another is still CALIBRATING.</t>
+        </is>
+      </c>
+      <c r="E73" s="10" t="inlineStr">
+        <is>
+          <t>Only the FINALISED (APPROVED/COMPLETED) reviews produce bonus items — the CALIBRATING review is excluded (pre-final ratings never reach compensation).</t>
+        </is>
+      </c>
+      <c r="F73" s="8" t="inlineStr"/>
+      <c r="G73" s="10" t="inlineStr"/>
+    </row>
   </sheetData>
   <dataValidations count="1">
-    <dataValidation sqref="F2:F60" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="F2:F73" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"Pass,Fail,Blocked,Not Run"</formula1>
     </dataValidation>
   </dataValidations>
@@ -2412,7 +2789,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="B1:E20"/>
+  <dimension ref="B1:E24"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="3" customWidth="1" min="1" max="1"/>
@@ -2554,30 +2931,70 @@
     <row r="14">
       <c r="B14" s="13" t="inlineStr">
         <is>
-          <t>Permissions (SEC)</t>
+          <t>PIPs (PIP)</t>
         </is>
       </c>
       <c r="C14" s="14" t="n"/>
       <c r="D14" s="15" t="n"/>
       <c r="E14" s="15" t="n"/>
     </row>
+    <row r="15">
+      <c r="B15" s="13" t="inlineStr">
+        <is>
+          <t>Development plans (DVP)</t>
+        </is>
+      </c>
+      <c r="C15" s="14" t="n"/>
+      <c r="D15" s="15" t="n"/>
+      <c r="E15" s="15" t="n"/>
+    </row>
+    <row r="16">
+      <c r="B16" s="13" t="inlineStr">
+        <is>
+          <t>Continuous feedback + check-ins (CFB/CIN)</t>
+        </is>
+      </c>
+      <c r="C16" s="14" t="n"/>
+      <c r="D16" s="15" t="n"/>
+      <c r="E16" s="15" t="n"/>
+    </row>
     <row r="17">
-      <c r="B17" s="16" t="inlineStr">
+      <c r="B17" s="13" t="inlineStr">
+        <is>
+          <t>Dashboard + notifications + comp guard (DSH/NTF/CMP-G)</t>
+        </is>
+      </c>
+      <c r="C17" s="14" t="n"/>
+      <c r="D17" s="15" t="n"/>
+      <c r="E17" s="15" t="n"/>
+    </row>
+    <row r="18">
+      <c r="B18" s="13" t="inlineStr">
+        <is>
+          <t>Permissions (SEC)</t>
+        </is>
+      </c>
+      <c r="C18" s="14" t="n"/>
+      <c r="D18" s="15" t="n"/>
+      <c r="E18" s="15" t="n"/>
+    </row>
+    <row r="21">
+      <c r="B21" s="16" t="inlineStr">
         <is>
           <t>Overall decision (SHIP / DON'T SHIP):</t>
         </is>
       </c>
-      <c r="C17" s="14" t="n"/>
-    </row>
-    <row r="19">
-      <c r="B19" s="17" t="inlineStr">
+      <c r="C21" s="14" t="n"/>
+    </row>
+    <row r="23">
+      <c r="B23" s="17" t="inlineStr">
         <is>
           <t>Tester name:</t>
         </is>
       </c>
     </row>
-    <row r="20">
-      <c r="B20" s="17" t="inlineStr">
+    <row r="24">
+      <c r="B24" s="17" t="inlineStr">
         <is>
           <t>Date:</t>
         </is>
@@ -2585,7 +3002,7 @@
     </row>
   </sheetData>
   <dataValidations count="1">
-    <dataValidation sqref="C4 C5 C6 C7 C8 C9 C10 C11 C12 C13 C14" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="C4 C5 C6 C7 C8 C9 C10 C11 C12 C13 C14 C15 C16 C17 C18" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"Pass,Fail,Blocked,Not Run"</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>